<commit_message>
Fix UNICEF VF project budget to exact USD 100,000
Co-authored-by: carbonintelli <carbonintelli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
+++ b/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
@@ -1282,14 +1282,8 @@
         </is>
       </c>
       <c r="B6" s="139" t="n"/>
-      <c r="C6" s="51">
-        <f>SUM(C7:C22)</f>
-        <v/>
-      </c>
-      <c r="D6" s="51">
-        <f>SUM(D7:D22)</f>
-        <v/>
-      </c>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="51" t="n"/>
     </row>
     <row r="7" ht="15.65" customHeight="1">
       <c r="A7" s="61" t="inlineStr">
@@ -1298,9 +1292,7 @@
         </is>
       </c>
       <c r="B7" s="50" t="n"/>
-      <c r="C7" s="105" t="n">
-        <v>2000</v>
-      </c>
+      <c r="C7" s="105" t="n"/>
       <c r="D7" s="105" t="n"/>
     </row>
     <row r="8" ht="15.65" customHeight="1">
@@ -1498,14 +1490,8 @@
         </is>
       </c>
       <c r="B23" s="141" t="n"/>
-      <c r="C23" s="51">
-        <f>SUM(C24:C39)</f>
-        <v/>
-      </c>
-      <c r="D23" s="51">
-        <f>SUM(D24:D39)</f>
-        <v/>
-      </c>
+      <c r="C23" s="51" t="n"/>
+      <c r="D23" s="51" t="n"/>
     </row>
     <row r="24" ht="15.65" customHeight="1">
       <c r="A24" s="61" t="inlineStr">
@@ -1706,14 +1692,8 @@
         </is>
       </c>
       <c r="B40" s="141" t="n"/>
-      <c r="C40" s="51">
-        <f>SUM(C41:C56)</f>
-        <v/>
-      </c>
-      <c r="D40" s="51">
-        <f>SUM(D41:D56)</f>
-        <v/>
-      </c>
+      <c r="C40" s="51" t="n"/>
+      <c r="D40" s="51" t="n"/>
     </row>
     <row r="41" ht="17.9" customHeight="1">
       <c r="A41" s="61" t="inlineStr">
@@ -1759,7 +1739,7 @@
         </is>
       </c>
       <c r="C43" s="105" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="D43" s="105" t="n"/>
     </row>
@@ -1914,14 +1894,8 @@
         </is>
       </c>
       <c r="B57" s="141" t="n"/>
-      <c r="C57" s="51">
-        <f>SUM(C58:C72)</f>
-        <v/>
-      </c>
-      <c r="D57" s="51">
-        <f>SUM(D58:D72)</f>
-        <v/>
-      </c>
+      <c r="C57" s="51" t="n"/>
+      <c r="D57" s="51" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="61" t="inlineStr">
@@ -1935,7 +1909,7 @@
         </is>
       </c>
       <c r="C58" s="105" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="D58" s="105" t="n"/>
     </row>
@@ -1967,7 +1941,7 @@
         </is>
       </c>
       <c r="C60" s="105" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="D60" s="105" t="n"/>
     </row>
@@ -2112,14 +2086,8 @@
     <row r="73" ht="18.5" customHeight="1">
       <c r="A73" s="4" t="n"/>
       <c r="B73" s="53" t="n"/>
-      <c r="C73" s="54">
-        <f>SUM(C6,C23,C40,C57)</f>
-        <v/>
-      </c>
-      <c r="D73" s="54">
-        <f>SUM(D6,D23,D40,D57)</f>
-        <v/>
-      </c>
+      <c r="C73" s="54" t="n"/>
+      <c r="D73" s="54" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="53" t="n"/>

</xml_diff>

<commit_message>
Optimize Template 7 budget toward pilots, PWA, and evidence
Reallocate USD 100k: Q1 22k, Q2 30k, Q3 28k, Q4 20k; cut low-leverage admin/spike spend.

Co-authored-by: carbonintelli <carbonintelli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
+++ b/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="C8" s="105" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="D8" s="105" t="n"/>
     </row>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="C9" s="105" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="D9" s="105" t="n"/>
     </row>
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="C12" s="105" t="n">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="D12" s="105" t="n"/>
     </row>
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="C13" s="105" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="D13" s="105" t="n"/>
     </row>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="C16" s="105" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="D16" s="105" t="n"/>
     </row>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="C21" s="105" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D21" s="105" t="n"/>
     </row>
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="C25" s="105" t="n">
-        <v>6000</v>
+        <v>7000</v>
       </c>
       <c r="D25" s="105" t="n"/>
     </row>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="C29" s="105" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="D29" s="105" t="n"/>
     </row>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C30" s="105" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D30" s="105" t="n"/>
     </row>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C33" s="105" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="D33" s="105" t="n"/>
     </row>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="C34" s="105" t="n">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="D34" s="105" t="n"/>
     </row>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B37" s="62" t="inlineStr">
         <is>
-          <t>DHIS2 interoperability spike</t>
+          <t>DHIS2 interoperability spike (lean)</t>
         </is>
       </c>
       <c r="C37" s="105" t="n">
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="C38" s="105" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D38" s="105" t="n"/>
     </row>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="C42" s="105" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="D42" s="105" t="n"/>
     </row>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="C43" s="105" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="D43" s="105" t="n"/>
     </row>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="C46" s="105" t="n">
-        <v>5000</v>
+        <v>5500</v>
       </c>
       <c r="D46" s="105" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="C47" s="105" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D47" s="105" t="n"/>
     </row>
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="C51" s="105" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D51" s="105" t="n"/>
     </row>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="C54" s="105" t="n">
-        <v>4000</v>
+        <v>4500</v>
       </c>
       <c r="D54" s="105" t="n"/>
     </row>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="C55" s="105" t="n">
-        <v>2000</v>
+        <v>3500</v>
       </c>
       <c r="D55" s="105" t="n"/>
     </row>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="C59" s="105" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="D59" s="105" t="n"/>
     </row>
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="C60" s="105" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="D60" s="105" t="n"/>
     </row>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="C64" s="105" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="D64" s="105" t="n"/>
     </row>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="C67" s="106" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="D67" s="106" t="n"/>
     </row>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="C68" s="106" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="D68" s="106" t="n"/>
     </row>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="C71" s="106" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="D71" s="106" t="n"/>
     </row>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="C72" s="106" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="D72" s="106" t="n"/>
     </row>

</xml_diff>

<commit_message>
Reduce UNGM VF budget request to USD 60,000
Lean Template 7 allocation (Q1 12k / Q2 20k / Q3 16k / Q4 12k); update bid references.

Co-authored-by: carbonintelli <carbonintelli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
+++ b/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="C8" s="105" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="D8" s="105" t="n"/>
     </row>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="C9" s="105" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D9" s="105" t="n"/>
     </row>
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="C12" s="105" t="n">
-        <v>4500</v>
+        <v>2500</v>
       </c>
       <c r="D12" s="105" t="n"/>
     </row>
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="C13" s="105" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="D13" s="105" t="n"/>
     </row>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="C16" s="105" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="D16" s="105" t="n"/>
     </row>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="C17" s="105" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="D17" s="105" t="n"/>
     </row>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="C20" s="105" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="D20" s="105" t="n"/>
     </row>
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="C21" s="105" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D21" s="105" t="n"/>
     </row>
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="C25" s="105" t="n">
-        <v>7000</v>
+        <v>4500</v>
       </c>
       <c r="D25" s="105" t="n"/>
     </row>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="C26" s="105" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="D26" s="105" t="n"/>
     </row>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="C29" s="105" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="D29" s="105" t="n"/>
     </row>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C30" s="105" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D30" s="105" t="n"/>
     </row>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C33" s="105" t="n">
-        <v>8000</v>
+        <v>6000</v>
       </c>
       <c r="D33" s="105" t="n"/>
     </row>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="C34" s="105" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="D34" s="105" t="n"/>
     </row>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="C37" s="105" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D37" s="105" t="n"/>
     </row>
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="C38" s="105" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D38" s="105" t="n"/>
     </row>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="C42" s="105" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="D42" s="105" t="n"/>
     </row>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="C43" s="105" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D43" s="105" t="n"/>
     </row>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="C46" s="105" t="n">
-        <v>5500</v>
+        <v>3500</v>
       </c>
       <c r="D46" s="105" t="n"/>
     </row>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="C47" s="105" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D47" s="105" t="n"/>
     </row>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="C50" s="105" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="D50" s="105" t="n"/>
     </row>
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="C51" s="105" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D51" s="105" t="n"/>
     </row>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="C54" s="105" t="n">
-        <v>4500</v>
+        <v>2000</v>
       </c>
       <c r="D54" s="105" t="n"/>
     </row>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="C55" s="105" t="n">
-        <v>3500</v>
+        <v>1500</v>
       </c>
       <c r="D55" s="105" t="n"/>
     </row>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="C59" s="105" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="D59" s="105" t="n"/>
     </row>
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="C60" s="105" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D60" s="105" t="n"/>
     </row>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="C63" s="105" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="D63" s="105" t="n"/>
     </row>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="C64" s="105" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D64" s="105" t="n"/>
     </row>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="C67" s="106" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D67" s="106" t="n"/>
     </row>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="C68" s="106" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D68" s="106" t="n"/>
     </row>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="C71" s="106" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D71" s="106" t="n"/>
     </row>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="C72" s="106" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D72" s="106" t="n"/>
     </row>
@@ -7907,7 +7907,7 @@
     <row r="2" ht="15.5" customHeight="1">
       <c r="A2" s="121" t="inlineStr">
         <is>
-          <t>Budget Period: January 20XX to December 20XX</t>
+          <t>Budget Period: September 2026 to August 2027</t>
         </is>
       </c>
       <c r="B2" s="142" t="n"/>
@@ -7917,7 +7917,7 @@
     <row r="3" ht="17.15" customHeight="1">
       <c r="A3" s="79" t="inlineStr">
         <is>
-          <t>Company Name:</t>
+          <t>Sustainow Technologies Private Limited</t>
         </is>
       </c>
       <c r="B3" s="143" t="inlineStr">
@@ -8125,9 +8125,17 @@
       </c>
     </row>
     <row r="17" ht="15.5" customHeight="1">
-      <c r="A17" s="67" t="n"/>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="19" t="n"/>
+      <c r="A17" s="67" t="inlineStr">
+        <is>
+          <t>UNICEF Venture Fund seed</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>30000</v>
+      </c>
       <c r="D17" s="91" t="n"/>
       <c r="E17" s="81" t="n"/>
       <c r="F17" s="81" t="n"/>

</xml_diff>

<commit_message>
Fill Template 7 Tab 2 company 1-year budget for USD 60k seed
Add H1/H2 income and expense lines in USD only; ETH left blank.

Co-authored-by: carbonintelli <carbonintelli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
+++ b/UNGM/submission/07_Budget_Proposal_Sustainow_KlimaGuardKids.xlsx
@@ -7917,7 +7917,7 @@
     <row r="3" ht="17.15" customHeight="1">
       <c r="A3" s="79" t="inlineStr">
         <is>
-          <t>Sustainow Technologies Private Limited</t>
+          <t>SUSTAINOW TECHNOLOGIES PRIVATE LIMITED</t>
         </is>
       </c>
       <c r="B3" s="143" t="inlineStr">
@@ -8013,18 +8013,34 @@
       </c>
     </row>
     <row r="7" ht="15.5" customHeight="1">
-      <c r="A7" s="67" t="n"/>
-      <c r="B7" s="19" t="n"/>
-      <c r="C7" s="19" t="n"/>
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>Pilot / implementation support revenue</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>5000</v>
+      </c>
       <c r="D7" s="91" t="n"/>
       <c r="E7" s="81" t="n"/>
       <c r="F7" s="81" t="n"/>
       <c r="G7" s="97" t="n"/>
     </row>
     <row r="8" ht="15.5" customHeight="1">
-      <c r="A8" s="67" t="n"/>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="19" t="n"/>
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>CSR / programme partnership fees</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>4000</v>
+      </c>
       <c r="D8" s="91" t="n"/>
       <c r="E8" s="81" t="n"/>
       <c r="F8" s="81" t="n"/>
@@ -8099,35 +8115,20 @@
           <t>Non-Operating Income [List detailed budget items in rows below (see example sheet for suggestions).</t>
         </is>
       </c>
-      <c r="B16" s="31">
-        <f>SUM(B17:B26)</f>
-        <v/>
-      </c>
-      <c r="C16" s="31">
-        <f>SUM(C17:C26)</f>
-        <v/>
-      </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
       <c r="D16" s="90">
         <f>SUM(B16:C16)</f>
         <v/>
       </c>
-      <c r="E16" s="80">
-        <f>SUM(E17:E26)</f>
-        <v/>
-      </c>
-      <c r="F16" s="80">
-        <f>SUM(F17:F26)</f>
-        <v/>
-      </c>
-      <c r="G16" s="96">
-        <f>SUM(E16:F16)</f>
-        <v/>
-      </c>
+      <c r="E16" s="80" t="n"/>
+      <c r="F16" s="80" t="n"/>
+      <c r="G16" s="96" t="n"/>
     </row>
     <row r="17" ht="15.5" customHeight="1">
       <c r="A17" s="67" t="inlineStr">
         <is>
-          <t>UNICEF Venture Fund seed</t>
+          <t>UNICEF Venture Fund seed (equity-free)</t>
         </is>
       </c>
       <c r="B17" s="19" t="n">
@@ -8142,9 +8143,17 @@
       <c r="G17" s="97" t="n"/>
     </row>
     <row r="18" ht="15.5" customHeight="1">
-      <c r="A18" s="67" t="n"/>
-      <c r="B18" s="19" t="n"/>
-      <c r="C18" s="19" t="n"/>
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>Founder capital contribution</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>4000</v>
+      </c>
       <c r="D18" s="91" t="n"/>
       <c r="E18" s="81" t="n"/>
       <c r="F18" s="81" t="n"/>
@@ -8228,30 +8237,15 @@
           <t>TOTAL INCOME</t>
         </is>
       </c>
-      <c r="B27" s="32">
-        <f>B6+B16</f>
-        <v/>
-      </c>
-      <c r="C27" s="32">
-        <f>C6+C16</f>
-        <v/>
-      </c>
+      <c r="B27" s="32" t="n"/>
+      <c r="C27" s="32" t="n"/>
       <c r="D27" s="32">
         <f>SUM(B27:C27)</f>
         <v/>
       </c>
-      <c r="E27" s="82">
-        <f>E6+E16</f>
-        <v/>
-      </c>
-      <c r="F27" s="82">
-        <f>F6+F16</f>
-        <v/>
-      </c>
-      <c r="G27" s="82">
-        <f>SUM(E27:F27)</f>
-        <v/>
-      </c>
+      <c r="E27" s="82" t="n"/>
+      <c r="F27" s="82" t="n"/>
+      <c r="G27" s="82" t="n"/>
     </row>
     <row r="28" ht="15.5" customFormat="1" customHeight="1" s="8">
       <c r="A28" s="70" t="n"/>
@@ -8265,83 +8259,151 @@
     <row r="29" ht="31" customFormat="1" customHeight="1" s="27">
       <c r="A29" s="33" t="inlineStr">
         <is>
-          <t>Expenses [List detailed budget items in rows below (see example sheet for suggestions).</t>
-        </is>
-      </c>
-      <c r="B29" s="28" t="n"/>
-      <c r="C29" s="28" t="n"/>
+          <t>Salaries &amp; director stipends (KlimaGuard Kids)</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C29" s="28" t="n">
+        <v>11000</v>
+      </c>
       <c r="D29" s="93" t="n"/>
       <c r="E29" s="84" t="n"/>
       <c r="F29" s="84" t="n"/>
       <c r="G29" s="99" t="n"/>
     </row>
     <row r="30" ht="15.5" customHeight="1">
-      <c r="A30" s="67" t="n"/>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
+      <c r="A30" s="67" t="inlineStr">
+        <is>
+          <t>Contractors (engineering, field facilitation, M&amp;E)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>8000</v>
+      </c>
       <c r="D30" s="91" t="n"/>
       <c r="E30" s="81" t="n"/>
       <c r="F30" s="81" t="n"/>
       <c r="G30" s="97" t="n"/>
     </row>
     <row r="31" ht="15.5" customHeight="1">
-      <c r="A31" s="67" t="n"/>
-      <c r="B31" s="19" t="n"/>
-      <c r="C31" s="19" t="n"/>
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>Cloud hosting, tooling &amp; CI</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C31" s="19" t="n">
+        <v>1000</v>
+      </c>
       <c r="D31" s="91" t="n"/>
       <c r="E31" s="81" t="n"/>
       <c r="F31" s="81" t="n"/>
       <c r="G31" s="97" t="n"/>
     </row>
     <row r="32" ht="15.5" customHeight="1">
-      <c r="A32" s="67" t="n"/>
-      <c r="B32" s="19" t="n"/>
-      <c r="C32" s="19" t="n"/>
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>Pilot travel &amp; CHW/school workshops</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C32" s="19" t="n">
+        <v>4500</v>
+      </c>
       <c r="D32" s="91" t="n"/>
       <c r="E32" s="81" t="n"/>
       <c r="F32" s="81" t="n"/>
       <c r="G32" s="97" t="n"/>
     </row>
     <row r="33" ht="15.5" customHeight="1">
-      <c r="A33" s="67" t="n"/>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="19" t="n"/>
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>Product hardening (PWA, i18n, content, a11y)</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C33" s="19" t="n">
+        <v>5000</v>
+      </c>
       <c r="D33" s="91" t="n"/>
       <c r="E33" s="81" t="n"/>
       <c r="F33" s="81" t="n"/>
       <c r="G33" s="97" t="n"/>
     </row>
     <row r="34" ht="15.5" customHeight="1">
-      <c r="A34" s="67" t="n"/>
-      <c r="B34" s="19" t="n"/>
-      <c r="C34" s="19" t="n"/>
+      <c r="A34" s="67" t="inlineStr">
+        <is>
+          <t>General &amp; administration</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>1500</v>
+      </c>
       <c r="D34" s="91" t="n"/>
       <c r="E34" s="81" t="n"/>
       <c r="F34" s="81" t="n"/>
       <c r="G34" s="97" t="n"/>
     </row>
     <row r="35" ht="15.5" customHeight="1">
-      <c r="A35" s="67" t="n"/>
-      <c r="B35" s="19" t="n"/>
-      <c r="C35" s="19" t="n"/>
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>Marketing &amp; open-source community</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C35" s="19" t="n">
+        <v>1500</v>
+      </c>
       <c r="D35" s="91" t="n"/>
       <c r="E35" s="81" t="n"/>
       <c r="F35" s="81" t="n"/>
       <c r="G35" s="97" t="n"/>
     </row>
     <row r="36" ht="15.5" customHeight="1">
-      <c r="A36" s="68" t="n"/>
-      <c r="B36" s="19" t="n"/>
-      <c r="C36" s="19" t="n"/>
+      <c r="A36" s="68" t="inlineStr">
+        <is>
+          <t>Legal, safeguarding &amp; privacy compliance</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C36" s="19" t="n">
+        <v>1500</v>
+      </c>
       <c r="D36" s="91" t="n"/>
       <c r="E36" s="81" t="n"/>
       <c r="F36" s="81" t="n"/>
       <c r="G36" s="97" t="n"/>
     </row>
     <row r="37" ht="15.5" customHeight="1">
-      <c r="A37" s="68" t="n"/>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
+      <c r="A37" s="68" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <v>500</v>
+      </c>
       <c r="D37" s="91" t="n"/>
       <c r="E37" s="81" t="n"/>
       <c r="F37" s="81" t="n"/>
@@ -8362,30 +8424,15 @@
           <t>TOTAL EXPENSE</t>
         </is>
       </c>
-      <c r="B39" s="32">
-        <f>SUM(B29:B38)</f>
-        <v/>
-      </c>
-      <c r="C39" s="32">
-        <f>SUM(C29:C38)</f>
-        <v/>
-      </c>
+      <c r="B39" s="32" t="n"/>
+      <c r="C39" s="32" t="n"/>
       <c r="D39" s="32">
         <f>SUM(B39:C39)</f>
         <v/>
       </c>
-      <c r="E39" s="82">
-        <f>SUM(E29:E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="82">
-        <f>SUM(F29:F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="82">
-        <f>SUM(E39:F39)</f>
-        <v/>
-      </c>
+      <c r="E39" s="82" t="n"/>
+      <c r="F39" s="82" t="n"/>
+      <c r="G39" s="82" t="n"/>
     </row>
     <row r="40" ht="15.5" customFormat="1" customHeight="1" s="8">
       <c r="A40" s="71" t="n"/>
@@ -8402,30 +8449,15 @@
           <t>Net Income Before Tax</t>
         </is>
       </c>
-      <c r="B41" s="18">
-        <f>B27-B39</f>
-        <v/>
-      </c>
-      <c r="C41" s="18">
-        <f>C27-C39</f>
-        <v/>
-      </c>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="18" t="n"/>
       <c r="D41" s="94">
         <f>D27-D39</f>
         <v/>
       </c>
-      <c r="E41" s="85">
-        <f>E27-E39</f>
-        <v/>
-      </c>
-      <c r="F41" s="85">
-        <f>F27-F39</f>
-        <v/>
-      </c>
-      <c r="G41" s="100">
-        <f>G27-G39</f>
-        <v/>
-      </c>
+      <c r="E41" s="85" t="n"/>
+      <c r="F41" s="85" t="n"/>
+      <c r="G41" s="100" t="n"/>
     </row>
     <row r="42" ht="14.5" customFormat="1" customHeight="1" s="26">
       <c r="A42" s="70" t="inlineStr">
@@ -8433,8 +8465,12 @@
           <t>Income Tax Expense</t>
         </is>
       </c>
-      <c r="B42" s="17" t="n"/>
-      <c r="C42" s="17" t="n"/>
+      <c r="B42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="D42" s="89" t="n"/>
       <c r="E42" s="86" t="n"/>
       <c r="F42" s="86" t="n"/>
@@ -8455,30 +8491,15 @@
           <t>NET INCOME</t>
         </is>
       </c>
-      <c r="B44" s="32">
-        <f>B41-B42</f>
-        <v/>
-      </c>
-      <c r="C44" s="32">
-        <f>C41-C42</f>
-        <v/>
-      </c>
+      <c r="B44" s="32" t="n"/>
+      <c r="C44" s="32" t="n"/>
       <c r="D44" s="32">
         <f>SUM(B44:C44)</f>
         <v/>
       </c>
-      <c r="E44" s="82">
-        <f>E41-E42</f>
-        <v/>
-      </c>
-      <c r="F44" s="82">
-        <f>F41-F42</f>
-        <v/>
-      </c>
-      <c r="G44" s="82">
-        <f>SUM(E44:F44)</f>
-        <v/>
-      </c>
+      <c r="E44" s="82" t="n"/>
+      <c r="F44" s="82" t="n"/>
+      <c r="G44" s="82" t="n"/>
     </row>
     <row r="45" ht="15.5" customHeight="1">
       <c r="A45" s="73" t="n"/>

</xml_diff>